<commit_message>
CBVG: corrige presentacion del filtro de Ano
- Estiliza #anioSelect igual que los otros (mismo alto/borde/radio, mas angosto).
- Agrupa etiqueta+lista (.fgrp) para que no se separen al hacer wrap.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CBVG/Tabla_puntos_evidencias_con_coordenadas (1).xlsx
+++ b/CBVG/Tabla_puntos_evidencias_con_coordenadas (1).xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\malej\OneDrive\Escritorio\IOT\GeoportalGRDGirardota\CBVG\Evidencia de Atencion\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\malej\OneDrive\Escritorio\IOT\GeoportalGRDGirardota\CBVG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A31B12BE-BAD0-46AC-B54B-77EECC2F07B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EF2D2CE-90E6-4B69-8115-380F7B82827B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,13 +17,25 @@
     <sheet name="OCR visible" sheetId="2" r:id="rId2"/>
     <sheet name="Notas" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
-  <fileRecoveryPr repairLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="232">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="245">
   <si>
     <t>Numeración</t>
   </si>
@@ -719,6 +731,45 @@
   </si>
   <si>
     <t>Las coordenadas no están como metadatos EXIF; se encuentran visibles/sobreimpresas en las fotografías. La tabla fue generada mediante lectura OCR y revisión visual de coordenadas visibles. Se recomienda validar los puntos que queden en blanco o con lectura parcial directamente contra la fotografía original.</t>
+  </si>
+  <si>
+    <t>SALUD EVENTO MASIVO</t>
+  </si>
+  <si>
+    <t>ATENCION PREHOSPITALARIA EN ACCIDENTE VIAL</t>
+  </si>
+  <si>
+    <t>ATENCION PREHOSPITALARIA</t>
+  </si>
+  <si>
+    <t>CONATO DE INCENDIO</t>
+  </si>
+  <si>
+    <t>RESCATE ANIMAL</t>
+  </si>
+  <si>
+    <t>ATENCION PREHOSPITALARIASALUD</t>
+  </si>
+  <si>
+    <t>INCENDIO ESTRUCTURAL</t>
+  </si>
+  <si>
+    <t>CRECIENTE SÚBITA</t>
+  </si>
+  <si>
+    <t>EVENTO MASIVO</t>
+  </si>
+  <si>
+    <t>MOVIMIENTO EN MASA</t>
+  </si>
+  <si>
+    <t>INUNDACIÓN</t>
+  </si>
+  <si>
+    <t>INSPECCION DE SEGURIDAD</t>
+  </si>
+  <si>
+    <t>INCENDENDIO INDUSTRIAL</t>
   </si>
 </sst>
 </file>
@@ -814,7 +865,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="TablaPuntos" displayName="TablaPuntos" ref="A1:E44">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="TablaPuntos" displayName="TablaPuntos" ref="A1:E47">
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Numeración"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Fecha"/>
@@ -990,7 +1041,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -1030,7 +1081,7 @@
         <v>-75.45581833</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>6</v>
+        <v>234</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -1047,7 +1098,7 @@
         <v>-75.442520000000002</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>6</v>
+        <v>234</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -1064,7 +1115,7 @@
         <v>-75.437759999999997</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>6</v>
+        <v>234</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -1081,7 +1132,7 @@
         <v>-75.44259778</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>8</v>
+        <v>241</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -1098,7 +1149,7 @@
         <v>-75.456654999999998</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>10</v>
+        <v>232</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -1115,7 +1166,7 @@
         <v>-75.466343330000001</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>14</v>
+        <v>233</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -1132,7 +1183,7 @@
         <v>-75.476128329999995</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>16</v>
+        <v>239</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -1149,7 +1200,7 @@
         <v>-75.445961670000003</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>14</v>
+        <v>233</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -1166,7 +1217,7 @@
         <v>-75.42841833</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>21</v>
+        <v>235</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -1183,7 +1234,7 @@
         <v>-75.442734999999999</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>17</v>
+        <v>236</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -1200,7 +1251,7 @@
         <v>-75.440646670000007</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>16</v>
+        <v>239</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -1251,7 +1302,7 @@
         <v>-75.449822900000001</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>28</v>
+        <v>237</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -1268,7 +1319,7 @@
         <v>-75.450356139999997</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>12</v>
+        <v>233</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -1285,7 +1336,7 @@
         <v>-75.447375230000006</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>6</v>
+        <v>234</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -1302,7 +1353,7 @@
         <v>-75.443055220000005</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>6</v>
+        <v>234</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -1336,7 +1387,7 @@
         <v>-75.446657549999998</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>12</v>
+        <v>233</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -1353,7 +1404,7 @@
         <v>-75.439637169999997</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>6</v>
+        <v>234</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -1370,7 +1421,7 @@
         <v>-75.450362119999994</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>12</v>
+        <v>233</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -1387,7 +1438,7 @@
         <v>-75.442014080000007</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>39</v>
+        <v>238</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -1404,7 +1455,7 @@
         <v>-75.441968590000002</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>41</v>
+        <v>238</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -1421,7 +1472,7 @@
         <v>-75.437135609999999</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>6</v>
+        <v>234</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -1455,7 +1506,7 @@
         <v>-75.469533279999993</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>12</v>
+        <v>233</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -1489,7 +1540,7 @@
         <v>-75.445238970000005</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>6</v>
+        <v>234</v>
       </c>
     </row>
     <row r="30" spans="1:5">
@@ -1506,7 +1557,7 @@
         <v>-75.444735690000002</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>6</v>
+        <v>234</v>
       </c>
     </row>
     <row r="31" spans="1:5">
@@ -1523,7 +1574,7 @@
         <v>-75.446165359999995</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>51</v>
+        <v>240</v>
       </c>
     </row>
     <row r="32" spans="1:5">
@@ -1562,7 +1613,7 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" s="2">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B34" s="7">
         <v>45402</v>
@@ -1591,7 +1642,7 @@
         <v>-75.445400000000006</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>51</v>
+        <v>240</v>
       </c>
     </row>
     <row r="36" spans="1:5">
@@ -1608,144 +1659,171 @@
         <v>-75.456100000000006</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>63</v>
+        <v>243</v>
       </c>
     </row>
     <row r="37" spans="1:5">
-      <c r="A37" s="2">
-        <v>60</v>
-      </c>
-      <c r="B37" s="7">
-        <v>45679</v>
-      </c>
-      <c r="C37" s="2">
-        <v>6.4085363900000001</v>
-      </c>
-      <c r="D37" s="2">
-        <v>-75.42958222</v>
-      </c>
-      <c r="E37" s="2" t="s">
-        <v>67</v>
-      </c>
+      <c r="A37" s="2"/>
+      <c r="B37" s="7"/>
+      <c r="C37" s="2"/>
+      <c r="D37" s="2"/>
+      <c r="E37" s="2"/>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" s="2">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="B38" s="7">
-        <v>45696</v>
+        <v>45679</v>
       </c>
       <c r="C38" s="2">
-        <v>6.3685216699999998</v>
+        <v>6.4085363900000001</v>
       </c>
       <c r="D38" s="2">
-        <v>-75.45525361</v>
+        <v>-75.42958222</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>74</v>
+        <v>238</v>
       </c>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="2">
-        <v>67</v>
-      </c>
-      <c r="B39" s="7">
-        <v>45832</v>
-      </c>
-      <c r="C39" s="2">
-        <v>6.3989750000000001</v>
-      </c>
-      <c r="D39" s="2">
-        <v>-75.465885560000004</v>
-      </c>
+        <v>61</v>
+      </c>
+      <c r="B39" s="7"/>
+      <c r="C39" s="2"/>
+      <c r="D39" s="2"/>
       <c r="E39" s="2" t="s">
-        <v>77</v>
+        <v>244</v>
       </c>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" s="2">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="B40" s="7">
-        <v>45800</v>
-      </c>
-      <c r="C40" s="2">
-        <v>6.3946922199999996</v>
-      </c>
-      <c r="D40" s="2">
-        <v>-75.487539170000005</v>
-      </c>
+        <v>45777</v>
+      </c>
+      <c r="C40" s="2"/>
+      <c r="D40" s="2"/>
       <c r="E40" s="2" t="s">
-        <v>79</v>
+        <v>242</v>
       </c>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="2">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="B41" s="7">
-        <v>46197</v>
+        <v>45696</v>
       </c>
       <c r="C41" s="2">
-        <v>6.3728186000000004</v>
+        <v>6.3685216699999998</v>
       </c>
       <c r="D41" s="2">
-        <v>-75.450518599999995</v>
+        <v>-75.45525361</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>8</v>
+        <v>239</v>
       </c>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" s="2">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B42" s="7">
-        <v>46206</v>
+        <v>45832</v>
       </c>
       <c r="C42" s="2">
-        <v>6.3878066599999999</v>
+        <v>6.3989750000000001</v>
       </c>
       <c r="D42" s="2">
-        <v>-75.449090530000007</v>
+        <v>-75.465885560000004</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>50</v>
+        <v>241</v>
       </c>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" s="2">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B43" s="7">
-        <v>46186</v>
+        <v>45800</v>
       </c>
       <c r="C43" s="2">
-        <v>6.3878066599999999</v>
+        <v>6.3946922199999996</v>
       </c>
       <c r="D43" s="2">
-        <v>-75.449090530000007</v>
+        <v>-75.487539170000005</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>66</v>
+        <v>240</v>
       </c>
     </row>
     <row r="44" spans="1:5">
       <c r="A44" s="2">
+        <v>69</v>
+      </c>
+      <c r="B44" s="7">
+        <v>46197</v>
+      </c>
+      <c r="C44" s="2">
+        <v>6.3728186000000004</v>
+      </c>
+      <c r="D44" s="2">
+        <v>-75.450518599999995</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5">
+      <c r="A45" s="2">
+        <v>70</v>
+      </c>
+      <c r="B45" s="7">
+        <v>46206</v>
+      </c>
+      <c r="C45" s="2">
+        <v>6.3878066599999999</v>
+      </c>
+      <c r="D45" s="2">
+        <v>-75.449090530000007</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5">
+      <c r="A46" s="2">
+        <v>71</v>
+      </c>
+      <c r="B46" s="7">
+        <v>46186</v>
+      </c>
+      <c r="C46" s="2">
+        <v>6.3878066599999999</v>
+      </c>
+      <c r="D46" s="2">
+        <v>-75.449090530000007</v>
+      </c>
+      <c r="E46" s="2"/>
+    </row>
+    <row r="47" spans="1:5">
+      <c r="A47" s="2">
         <v>72</v>
       </c>
-      <c r="B44" s="7">
+      <c r="B47" s="7">
         <v>46187</v>
       </c>
-      <c r="C44" s="2">
+      <c r="C47" s="2">
         <v>6.38718611</v>
       </c>
-      <c r="D44" s="2">
+      <c r="D47" s="2">
         <v>-75.449536859999995</v>
       </c>
-      <c r="E44" s="2" t="s">
-        <v>66</v>
-      </c>
+      <c r="E47" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>